<commit_message>
Université Le Havre Normandie : périmètre élargi Le Havre et sa région (15 lycées)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reseau-lycees-le-havre.xlsx
+++ b/reseau-lycees-le-havre.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lycées Le Havre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Lycées Le Havre et région" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lycées Le Havre'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lycées Le Havre et région'!$A$1:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -76,18 +76,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,20 +464,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Région</t>
@@ -506,6 +517,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Effectifs approx.</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Distance du Havre (km)</t>
         </is>
       </c>
     </row>
@@ -525,7 +541,7 @@
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>76600</t>
         </is>
@@ -540,7 +556,7 @@
           <t>Lycée François Ier</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Général - Cpge - Littéraires et économiques - Lycée historique</t>
         </is>
@@ -548,45 +564,51 @@
       <c r="H2" s="3" t="n">
         <v>1400</v>
       </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Normandie</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Seine-Maritime</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>76600</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>35 Rue De La Victoire</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Lycée Privé Jeanne D'Arc</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Général - Sections européennes - Cadre de proximité et accompagnement personnalisé</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="6" t="n">
         <v>750</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -605,7 +627,7 @@
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>76600</t>
         </is>
@@ -620,7 +642,7 @@
           <t>Lycée Privé Saint-Joseph</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Général - Techno - St2s - Sections européennes - Suivi d'excellence</t>
         </is>
@@ -628,45 +650,51 @@
       <c r="H4" s="3" t="n">
         <v>900</v>
       </c>
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Normandie</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Seine-Maritime</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>76600</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Rue De La Mailleraye</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Lycée Professionnel Jules Siegfried</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Pro - De la logistique - Commerce</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="6" t="n">
         <v>550</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -685,7 +713,7 @@
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>76600</t>
         </is>
@@ -700,7 +728,7 @@
           <t>Lycée Professionnel Maritime Du Havre</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Pro - Conduite de navires - Mécanique marine - Cultures marines)</t>
         </is>
@@ -708,49 +736,442 @@
       <c r="H6" s="3" t="n">
         <v>400</v>
       </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Normandie</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Seine-Maritime</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>76600</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>15 Rue Robert Schuman</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Lycée Robert Schuman</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Général - Techno - Pro - Cpge</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="6" t="n">
         <v>1250</v>
       </c>
+      <c r="I7" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Eure</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Pont-Audemer</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>27500</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>6 Avenue De L'Europe</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Lycée Jacques Prévert</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Général - Techno - Sections européennes - Théâtre</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>850</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Eure</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Pont-Audemer</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>27500</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Route De Saint-Paul</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Risle-Seine</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Pro - Métallurgie - Maintenance - Électricité)</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Calvados</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Lisieux</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>14100</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>18 Rue De La Gare</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Lycée Marcel Gambier</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Général - Sections européennes - Théâtre</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Calvados</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Lisieux</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>14100</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>9 Rue Paul Cornu</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Lycée Paul Cornu</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Général - Techno - Pro</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>1100</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Calvados</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Lisieux</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>14100</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Avenue De La Basilique</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Lycée Privé Les Rosiers</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Techno - Social - Services aux personnes)</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Calvados</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Douvres-La-Délivrande</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>14440</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Route De Caen</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Lycée Privé Les Tourelles</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Général - Cadre d'excellence - Section sport et langues</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Calvados</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Mézidon Vallée D'Auge</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>14170</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Le Robillard</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Agricole Le Robillard</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Agricole (bac pro cgea - Stav - Bts agroéquipement - Aménagements paysagers)</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Eure</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Bernay</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>27300</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Rue De La Sous-Préfecture</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Lycée Privé Jeanne D'Arc</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Général - Effectifs à taille humaine - Encadrement méthodologique</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Eure</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Bernay</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>27300</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Rue Du Repos</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Clément Ader</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Pro - De l'usinage - Maintenance</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>380</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>57</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:I16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>